<commit_message>
Added datasheets for to-be-ordered components, double checked BOM
</commit_message>
<xml_diff>
--- a/ANE21_PCB.csv.xlsx
+++ b/ANE21_PCB.csv.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koeki\Documents\GitHub\ANE21_PCB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B80DEF26-4B08-4C66-A94C-342559C90DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E74F11-AF53-479F-96A4-5827AF862468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17280" windowHeight="8988" xr2:uid="{3B488360-DCDD-43B7-9EB7-515A94F904FC}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="41472" windowHeight="16752" xr2:uid="{3B488360-DCDD-43B7-9EB7-515A94F904FC}"/>
   </bookViews>
   <sheets>
     <sheet name="ANE21_PCB" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="120">
   <si>
     <t>Reference</t>
   </si>
@@ -308,6 +310,78 @@
   </si>
   <si>
     <t>Van school</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>PCIe connector</t>
+  </si>
+  <si>
+    <t>USB A</t>
+  </si>
+  <si>
+    <t>CM4</t>
+  </si>
+  <si>
+    <t>HDMI connector</t>
+  </si>
+  <si>
+    <t>DF40C-100DS-0.4V(51)</t>
+  </si>
+  <si>
+    <t>CM4 header</t>
+  </si>
+  <si>
+    <t>HDMI Load switch</t>
+  </si>
+  <si>
+    <t>FabrikantNr</t>
+  </si>
+  <si>
+    <t>10029449-111RLF</t>
+  </si>
+  <si>
+    <t>MCWR06X3322FTL</t>
+  </si>
+  <si>
+    <t>MCMR06X3162FTL</t>
+  </si>
+  <si>
+    <t>1255AY-3R3N=P3</t>
+  </si>
+  <si>
+    <t>GRM21BR71A106KA73L</t>
+  </si>
+  <si>
+    <t>CL10B104KO8NNNC</t>
+  </si>
+  <si>
+    <t>CL31B226KPHNNNE</t>
+  </si>
+  <si>
+    <t>DC-DC converter</t>
+  </si>
+  <si>
+    <t>33.2k R</t>
+  </si>
+  <si>
+    <t>31.6k R</t>
+  </si>
+  <si>
+    <t>3.3uH L</t>
+  </si>
+  <si>
+    <t>10 uF C</t>
+  </si>
+  <si>
+    <t>0.1uF C</t>
+  </si>
+  <si>
+    <t>22 uF C</t>
+  </si>
+  <si>
+    <t>Geplaatst</t>
   </si>
 </sst>
 </file>
@@ -1735,5 +1809,401 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92AC0A09-AEC2-49C8-AC02-0A0B2E44BCD4}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960A2C18-4BE4-42CD-A3BF-42E852C484EA}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="84.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="79" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>100</v>
+      </c>
+      <c r="D15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>103</v>
+      </c>
+      <c r="D16" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>